<commit_message>
ATENÇÃO REFATORAÇÃO SCRIPTS, reduzindo o tamanho monolitico dos scripts python
</commit_message>
<xml_diff>
--- a/projetos/OBRA_TMULT/06_SST_E_RH/HISTOGRAMA_MAO_DE_OBRA_TMULT.xlsx
+++ b/projetos/OBRA_TMULT/06_SST_E_RH/HISTOGRAMA_MAO_DE_OBRA_TMULT.xlsx
@@ -16,11 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="#,##0&quot; HH&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,19 +56,8 @@
       <color rgb="001B365D"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001B365D"/>
-      <sz val="12"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -102,18 +90,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8EEF5"/>
-        <bgColor rgb="00E8EEF5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C2D7EF"/>
-        <bgColor rgb="00C2D7EF"/>
+        <fgColor rgb="00E6F4EA"/>
+        <bgColor rgb="00E6F4EA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -135,11 +117,25 @@
         <color rgb="00DDDDDD"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00DDDDDD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001B365D"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -162,12 +158,6 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -180,32 +170,25 @@
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -572,27 +555,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TMULT — HISTOGRAMA OFICIAL DE MÃO DE OBRA &amp; HEADCOUNT MENSAL</t>
+          <t>TMULT — HISTOGRAMA DE MÃO DE OBRA &amp; HEADCOUNT MENSAL</t>
         </is>
       </c>
     </row>
@@ -600,7 +581,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Planejamento Físico de Efetivo | Total da Obra: 102 Headcount-Mês | 22,440 Horas-Homem (HH) | Carga Horária Padrão: 220 HH / mês</t>
+          <t>Planejamento Físico de Efetivo | 6 Meses (180 Dias) | Carga Horária Padrão: 220 Horas-Homem (HH) / mês</t>
         </is>
       </c>
     </row>
@@ -655,16 +636,6 @@
           <t>Mês 6</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Total Meses</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>Total Horas-Homem (HH)</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -703,55 +674,43 @@
       <c r="J6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="L6" s="9" t="n">
-        <v>1320</v>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Gestão</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Mestre de Obras Geral (100%)</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Mensalista</t>
         </is>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="10" t="n">
         <v>7120</v>
       </c>
-      <c r="E7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="L7" s="15" t="n">
-        <v>1320</v>
+      <c r="E7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -791,55 +750,43 @@
       <c r="J8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="K8" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="L8" s="9" t="n">
-        <v>1320</v>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>SST / Apoio</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Almoxarife / Apontador de Campo</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Mensalista</t>
         </is>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="10" t="n">
         <v>3500</v>
       </c>
-      <c r="E9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="L9" s="15" t="n">
-        <v>1320</v>
+      <c r="E9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -879,55 +826,43 @@
       <c r="J10" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="K10" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="L10" s="9" t="n">
-        <v>1320</v>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Produção</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Pedreiro Oficial (Alvenaria / Reboco)</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Horista/Produção</t>
         </is>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="10" t="n">
         <v>3200</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="13" t="n">
+      <c r="G11" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="13" t="n">
+      <c r="H11" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="14" t="n">
-        <v>13</v>
-      </c>
-      <c r="L11" s="15" t="n">
-        <v>2860</v>
+      <c r="I11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -967,55 +902,43 @@
       <c r="J12" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="L12" s="9" t="n">
-        <v>660</v>
-      </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Produção</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Carpinteiro de Fôrmas e Escoramento</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Horista/Produção</t>
         </is>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="10" t="n">
         <v>3200</v>
       </c>
-      <c r="E13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="13" t="n">
+      <c r="E13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" s="15" t="n">
-        <v>880</v>
+      <c r="G13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1055,55 +978,43 @@
       <c r="J14" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L14" s="9" t="n">
-        <v>1100</v>
-      </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Produção</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Montador de Estrutura Metálica / Telhadista</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Especialista</t>
         </is>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="10" t="n">
         <v>3600</v>
       </c>
-      <c r="E15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="13" t="n">
+      <c r="E15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="L15" s="15" t="n">
-        <v>660</v>
+      <c r="H15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1143,55 +1054,43 @@
       <c r="J16" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="K16" s="8" t="n">
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Produção</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Servente de Obras / Ajudante Prático</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Horista/Produção</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>2200</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="L16" s="9" t="n">
-        <v>1100</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>Produção</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Servente de Obras / Ajudante Prático</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>Horista/Produção</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="n">
-        <v>2200</v>
-      </c>
-      <c r="E17" s="13" t="n">
+      <c r="G17" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="G17" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="H17" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="I17" s="13" t="n">
+      <c r="I17" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="J17" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="14" t="n">
-        <v>21</v>
-      </c>
-      <c r="L17" s="15" t="n">
-        <v>4620</v>
+      <c r="J17" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1231,55 +1130,43 @@
       <c r="J18" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="K18" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L18" s="9" t="n">
-        <v>1100</v>
-      </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Instalações</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Encanador / Bombeiro Hidráulico</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Oficial</t>
         </is>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="10" t="n">
         <v>3300</v>
       </c>
-      <c r="E19" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="13" t="n">
+      <c r="E19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="I19" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="L19" s="15" t="n">
-        <v>880</v>
+      <c r="I19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1319,55 +1206,43 @@
       <c r="J20" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="K20" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="L20" s="9" t="n">
-        <v>880</v>
-      </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Instalações</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Marceneiro / Montador de Esquadrias</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Oficial</t>
         </is>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="10" t="n">
         <v>3200</v>
       </c>
-      <c r="E21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="13" t="n">
+      <c r="E21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="J21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" s="15" t="n">
-        <v>440</v>
+      <c r="J21" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1407,133 +1282,113 @@
       <c r="J22" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="9" t="n">
-        <v>220</v>
-      </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Apoio</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Auxiliar de Limpeza Especializada Pós-Obra</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Apoio</t>
         </is>
       </c>
-      <c r="D23" s="12" t="n">
+      <c r="D23" s="10" t="n">
         <v>2100</v>
       </c>
-      <c r="E23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="13" t="n">
+      <c r="E23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="K23" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" s="15" t="n">
-        <v>440</v>
-      </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>HEADCOUNT TOTAL DE CAMPO (Operários + Gestão)</t>
         </is>
       </c>
-      <c r="E24" s="18" t="n">
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="F24" s="18" t="n">
+      <c r="F24" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="G24" s="18" t="n">
+      <c r="G24" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="H24" s="18" t="n">
+      <c r="H24" s="15" t="n">
         <v>17</v>
       </c>
-      <c r="I24" s="18" t="n">
+      <c r="I24" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="J24" s="18" t="n">
+      <c r="J24" s="15" t="n">
         <v>16</v>
-      </c>
-      <c r="K24" s="18" t="n">
-        <v>102</v>
-      </c>
-      <c r="L24" s="19" t="n">
-        <v>22440</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>TOTAL HH</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>TOTAL DE HORAS-HOMEM PREVISTAS (HH/mês)</t>
-        </is>
-      </c>
-      <c r="E25" s="20" t="n">
+          <t>TOTAL DE HORAS-HOMEM PREVISTAS (220h / profissional)</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="19" t="n">
         <v>3080</v>
       </c>
-      <c r="F25" s="20" t="n">
+      <c r="F25" s="19" t="n">
         <v>4180</v>
       </c>
-      <c r="G25" s="20" t="n">
+      <c r="G25" s="19" t="n">
         <v>4400</v>
       </c>
-      <c r="H25" s="20" t="n">
+      <c r="H25" s="19" t="n">
         <v>3740</v>
       </c>
-      <c r="I25" s="20" t="n">
+      <c r="I25" s="19" t="n">
         <v>3520</v>
       </c>
-      <c r="J25" s="20" t="n">
+      <c r="J25" s="19" t="n">
         <v>3520</v>
-      </c>
-      <c r="K25" s="21" t="n">
-        <v>102</v>
-      </c>
-      <c r="L25" s="22" t="n">
-        <v>22440</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="A1:J2"/>
+    <mergeCell ref="A3:J3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ATENÇÃO FASE 4 - SCRIPT CRNOGRAM SUPRIMENTOS E CONTRATAÇÃO
</commit_message>
<xml_diff>
--- a/projetos/OBRA_TMULT/06_SST_E_RH/HISTOGRAMA_MAO_DE_OBRA_TMULT.xlsx
+++ b/projetos/OBRA_TMULT/06_SST_E_RH/HISTOGRAMA_MAO_DE_OBRA_TMULT.xlsx
@@ -16,11 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="#,##0&quot; HH&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,14 +56,8 @@
       <color rgb="001B365D"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001B365D"/>
-      <sz val="12"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -97,18 +90,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8EEF5"/>
-        <bgColor rgb="00E8EEF5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C2D7EF"/>
-        <bgColor rgb="00C2D7EF"/>
+        <fgColor rgb="00E6F4EA"/>
+        <bgColor rgb="00E6F4EA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -130,80 +117,78 @@
         <color rgb="00DDDDDD"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00DDDDDD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001B365D"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -570,35 +555,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TMULT — HISTOGRAMA OFICIAL DE MÃO DE OBRA &amp; HEADCOUNT MENSAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="2" customHeight="1"/>
+          <t>TMULT — HISTOGRAMA DE MÃO DE OBRA &amp; HEADCOUNT MENSAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Planejamento Físico de Efetivo | Total da Obra: 102 Headcount-Mês | 22,440 Horas-Homem (HH) | Carga Horária Padrão: 220 HH / mês</t>
+          <t>Planejamento Físico de Efetivo | 6 Meses (180 Dias) | Carga Horária Padrão: 220 Horas-Homem (HH) / mês</t>
         </is>
       </c>
     </row>
@@ -653,16 +636,6 @@
           <t>Mês 6</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Total Meses</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>Total Horas-Homem (HH)</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -701,55 +674,43 @@
       <c r="J6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="L6" s="9" t="n">
-        <v>1320</v>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Gestão</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Mestre de Obras Geral (100%)</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Mensalista</t>
         </is>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="10" t="n">
         <v>7120</v>
       </c>
-      <c r="E7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="L7" s="15" t="n">
-        <v>1320</v>
+      <c r="E7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -789,55 +750,43 @@
       <c r="J8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="K8" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="L8" s="9" t="n">
-        <v>1320</v>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>SST / Apoio</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Almoxarife / Apontador de Campo</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Mensalista</t>
         </is>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="10" t="n">
         <v>3500</v>
       </c>
-      <c r="E9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="L9" s="15" t="n">
-        <v>1320</v>
+      <c r="E9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -877,55 +826,43 @@
       <c r="J10" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="K10" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="L10" s="9" t="n">
-        <v>1320</v>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Produção</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Pedreiro Oficial (Alvenaria / Reboco)</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Horista/Produção</t>
         </is>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="10" t="n">
         <v>3200</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="13" t="n">
+      <c r="G11" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="13" t="n">
+      <c r="H11" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="14" t="n">
-        <v>13</v>
-      </c>
-      <c r="L11" s="15" t="n">
-        <v>2860</v>
+      <c r="I11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -965,55 +902,43 @@
       <c r="J12" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="L12" s="9" t="n">
-        <v>660</v>
-      </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Produção</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Carpinteiro de Fôrmas e Escoramento</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Horista/Produção</t>
         </is>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="10" t="n">
         <v>3200</v>
       </c>
-      <c r="E13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="13" t="n">
+      <c r="E13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" s="15" t="n">
-        <v>880</v>
+      <c r="G13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1053,55 +978,43 @@
       <c r="J14" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L14" s="9" t="n">
-        <v>1100</v>
-      </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Produção</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Montador de Estrutura Metálica / Telhadista</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Especialista</t>
         </is>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="10" t="n">
         <v>3600</v>
       </c>
-      <c r="E15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="13" t="n">
+      <c r="E15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="L15" s="15" t="n">
-        <v>660</v>
+      <c r="H15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1141,55 +1054,43 @@
       <c r="J16" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="K16" s="8" t="n">
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Produção</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Servente de Obras / Ajudante Prático</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Horista/Produção</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>2200</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="L16" s="9" t="n">
-        <v>1100</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>Produção</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Servente de Obras / Ajudante Prático</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>Horista/Produção</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="n">
-        <v>2200</v>
-      </c>
-      <c r="E17" s="13" t="n">
+      <c r="G17" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="G17" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="H17" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="I17" s="13" t="n">
+      <c r="I17" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="J17" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="14" t="n">
-        <v>21</v>
-      </c>
-      <c r="L17" s="15" t="n">
-        <v>4620</v>
+      <c r="J17" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1229,55 +1130,43 @@
       <c r="J18" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="K18" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L18" s="9" t="n">
-        <v>1100</v>
-      </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Instalações</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Encanador / Bombeiro Hidráulico</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Oficial</t>
         </is>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="10" t="n">
         <v>3300</v>
       </c>
-      <c r="E19" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="13" t="n">
+      <c r="E19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="I19" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="L19" s="15" t="n">
-        <v>880</v>
+      <c r="I19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1317,55 +1206,43 @@
       <c r="J20" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="K20" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="L20" s="9" t="n">
-        <v>880</v>
-      </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Instalações</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Marceneiro / Montador de Esquadrias</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Oficial</t>
         </is>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="10" t="n">
         <v>3200</v>
       </c>
-      <c r="E21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="13" t="n">
+      <c r="E21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="J21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" s="15" t="n">
-        <v>440</v>
+      <c r="J21" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1405,133 +1282,113 @@
       <c r="J22" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="9" t="n">
-        <v>220</v>
-      </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Apoio</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Auxiliar de Limpeza Especializada Pós-Obra</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Apoio</t>
         </is>
       </c>
-      <c r="D23" s="12" t="n">
+      <c r="D23" s="10" t="n">
         <v>2100</v>
       </c>
-      <c r="E23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="13" t="n">
+      <c r="E23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="K23" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" s="15" t="n">
-        <v>440</v>
-      </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>HEADCOUNT TOTAL DE CAMPO (Operários + Gestão)</t>
         </is>
       </c>
-      <c r="E24" s="18" t="n">
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="F24" s="18" t="n">
+      <c r="F24" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="G24" s="18" t="n">
+      <c r="G24" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="H24" s="18" t="n">
+      <c r="H24" s="15" t="n">
         <v>17</v>
       </c>
-      <c r="I24" s="18" t="n">
+      <c r="I24" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="J24" s="18" t="n">
+      <c r="J24" s="15" t="n">
         <v>16</v>
-      </c>
-      <c r="K24" s="19" t="n">
-        <v>102</v>
-      </c>
-      <c r="L24" s="20" t="n">
-        <v>22440</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>TOTAL HH</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>TOTAL DE HORAS-HOMEM PREVISTAS (HH/mês)</t>
-        </is>
-      </c>
-      <c r="E25" s="21" t="n">
+          <t>TOTAL DE HORAS-HOMEM PREVISTAS (220h / profissional)</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="19" t="n">
         <v>3080</v>
       </c>
-      <c r="F25" s="21" t="n">
+      <c r="F25" s="19" t="n">
         <v>4180</v>
       </c>
-      <c r="G25" s="21" t="n">
+      <c r="G25" s="19" t="n">
         <v>4400</v>
       </c>
-      <c r="H25" s="21" t="n">
+      <c r="H25" s="19" t="n">
         <v>3740</v>
       </c>
-      <c r="I25" s="21" t="n">
+      <c r="I25" s="19" t="n">
         <v>3520</v>
       </c>
-      <c r="J25" s="21" t="n">
+      <c r="J25" s="19" t="n">
         <v>3520</v>
-      </c>
-      <c r="K25" s="22" t="n">
-        <v>102</v>
-      </c>
-      <c r="L25" s="23" t="n">
-        <v>22440</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="A1:J2"/>
+    <mergeCell ref="A3:J3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(cronograma): sincroniza aceleracao e histograma multiobra
</commit_message>
<xml_diff>
--- a/projetos/OBRA_TMULT/06_SST_E_RH/HISTOGRAMA_MAO_DE_OBRA_TMULT.xlsx
+++ b/projetos/OBRA_TMULT/06_SST_E_RH/HISTOGRAMA_MAO_DE_OBRA_TMULT.xlsx
@@ -16,10 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="#,##0&quot; HH&quot;"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,8 +57,14 @@
       <color rgb="001B365D"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B365D"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -90,12 +97,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E6F4EA"/>
-        <bgColor rgb="00E6F4EA"/>
+        <fgColor rgb="00E8EEF5"/>
+        <bgColor rgb="00E8EEF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C2D7EF"/>
+        <bgColor rgb="00C2D7EF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -117,78 +130,80 @@
         <color rgb="00DDDDDD"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00DDDDDD"/>
-      </left>
-      <right style="thin">
-        <color rgb="00DDDDDD"/>
-      </right>
-      <top style="thin">
-        <color rgb="00DDDDDD"/>
-      </top>
-      <bottom style="double">
-        <color rgb="001B365D"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -555,33 +570,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TMULT — HISTOGRAMA DE MÃO DE OBRA &amp; HEADCOUNT MENSAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>TMULT — HISTOGRAMA OFICIAL DE MÃO DE OBRA &amp; HEADCOUNT MENSAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="2" customHeight="1"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Planejamento Físico de Efetivo | 6 Meses (180 Dias) | Carga Horária Padrão: 220 Horas-Homem (HH) / mês</t>
+          <t>Planejamento Físico de Efetivo | Total da Obra: 102 Headcount-Mês | 22,440 Horas-Homem (HH) | Carga Horária Padrão: 220 HH / mês</t>
         </is>
       </c>
     </row>
@@ -636,6 +653,16 @@
           <t>Mês 6</t>
         </is>
       </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Total Meses</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Total Horas-Homem (HH)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -674,43 +701,55 @@
       <c r="J6" s="7" t="n">
         <v>1</v>
       </c>
+      <c r="K6" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>1320</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Gestão</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Mestre de Obras Geral (100%)</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Mensalista</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="12" t="n">
         <v>7120</v>
       </c>
-      <c r="E7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="11" t="n">
-        <v>1</v>
+      <c r="E7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" s="15" t="n">
+        <v>1320</v>
       </c>
     </row>
     <row r="8">
@@ -750,43 +789,55 @@
       <c r="J8" s="7" t="n">
         <v>1</v>
       </c>
+      <c r="K8" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>1320</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>SST / Apoio</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Almoxarife / Apontador de Campo</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Mensalista</t>
         </is>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="12" t="n">
         <v>3500</v>
       </c>
-      <c r="E9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="11" t="n">
-        <v>1</v>
+      <c r="E9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="L9" s="15" t="n">
+        <v>1320</v>
       </c>
     </row>
     <row r="10">
@@ -826,43 +877,55 @@
       <c r="J10" s="7" t="n">
         <v>1</v>
       </c>
+      <c r="K10" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>1320</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Produção</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Pedreiro Oficial (Alvenaria / Reboco)</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Horista/Produção</t>
         </is>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="12" t="n">
         <v>3200</v>
       </c>
-      <c r="E11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G11" s="11" t="n">
+      <c r="E11" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="11" t="n">
-        <v>0</v>
+      <c r="I11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="L11" s="15" t="n">
+        <v>2420</v>
       </c>
     </row>
     <row r="12">
@@ -894,51 +957,63 @@
         <v>0</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>0</v>
       </c>
+      <c r="K12" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>1320</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Produção</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Carpinteiro de Fôrmas e Escoramento</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>Horista/Produção</t>
         </is>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="12" t="n">
         <v>3200</v>
       </c>
-      <c r="E13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="11" t="n">
-        <v>0</v>
+      <c r="E13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" s="15" t="n">
+        <v>440</v>
       </c>
     </row>
     <row r="14">
@@ -961,60 +1036,72 @@
         <v>3200</v>
       </c>
       <c r="E14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="G14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>0</v>
+      <c r="L14" s="9" t="n">
+        <v>660</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Produção</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Montador de Estrutura Metálica / Telhadista</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Especialista</t>
         </is>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="12" t="n">
         <v>3600</v>
       </c>
-      <c r="E15" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="H15" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="11" t="n">
-        <v>0</v>
+      <c r="E15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" s="15" t="n">
+        <v>440</v>
       </c>
     </row>
     <row r="16">
@@ -1049,48 +1136,60 @@
         <v>0</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>4</v>
       </c>
+      <c r="K16" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="L16" s="9" t="n">
+        <v>1760</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Produção</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Servente de Obras / Ajudante Prático</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Horista/Produção</t>
         </is>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D17" s="12" t="n">
         <v>2200</v>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="I17" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="G17" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J17" s="11" t="n">
-        <v>1</v>
+      <c r="K17" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="L17" s="15" t="n">
+        <v>5500</v>
       </c>
     </row>
     <row r="18">
@@ -1122,51 +1221,63 @@
         <v>1</v>
       </c>
       <c r="H18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I18" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="7" t="n">
-        <v>1</v>
+      <c r="K18" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L18" s="9" t="n">
+        <v>1100</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Instalações</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Encanador / Bombeiro Hidráulico</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>Oficial</t>
         </is>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="D19" s="12" t="n">
         <v>3300</v>
       </c>
-      <c r="E19" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="11" t="n">
+      <c r="E19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="I19" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="11" t="n">
-        <v>1</v>
+      <c r="L19" s="15" t="n">
+        <v>440</v>
       </c>
     </row>
     <row r="20">
@@ -1201,48 +1312,60 @@
         <v>0</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>2</v>
       </c>
+      <c r="K20" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="L20" s="9" t="n">
+        <v>660</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Instalações</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Marceneiro / Montador de Esquadrias</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Oficial</t>
         </is>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D21" s="12" t="n">
         <v>3200</v>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J21" s="11" t="n">
-        <v>0</v>
+      <c r="E21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" s="15" t="n">
+        <v>220</v>
       </c>
     </row>
     <row r="22">
@@ -1265,7 +1388,7 @@
         <v>3600</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" s="7" t="n">
         <v>0</v>
@@ -1282,113 +1405,133 @@
       <c r="J22" s="7" t="n">
         <v>0</v>
       </c>
+      <c r="K22" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Apoio</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Auxiliar de Limpeza Especializada Pós-Obra</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
         <is>
           <t>Apoio</t>
         </is>
       </c>
-      <c r="D23" s="10" t="n">
+      <c r="D23" s="12" t="n">
         <v>2100</v>
       </c>
-      <c r="E23" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="11" t="n">
-        <v>2</v>
+      <c r="E23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K23" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="L23" s="15" t="n">
+        <v>880</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>HEADCOUNT TOTAL DE CAMPO (Operários + Gestão)</t>
         </is>
       </c>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="15" t="n">
-        <v>14</v>
-      </c>
-      <c r="F24" s="15" t="n">
-        <v>19</v>
-      </c>
-      <c r="G24" s="15" t="n">
-        <v>20</v>
-      </c>
-      <c r="H24" s="15" t="n">
+      <c r="E24" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="F24" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="G24" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="H24" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="I24" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="I24" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="J24" s="15" t="n">
-        <v>16</v>
+      <c r="J24" s="18" t="n">
+        <v>22</v>
+      </c>
+      <c r="K24" s="19" t="n">
+        <v>102</v>
+      </c>
+      <c r="L24" s="20" t="n">
+        <v>22440</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>TOTAL HH</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>TOTAL DE HORAS-HOMEM PREVISTAS (220h / profissional)</t>
-        </is>
-      </c>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="18" t="n"/>
-      <c r="E25" s="19" t="n">
-        <v>3080</v>
-      </c>
-      <c r="F25" s="19" t="n">
-        <v>4180</v>
-      </c>
-      <c r="G25" s="19" t="n">
-        <v>4400</v>
-      </c>
-      <c r="H25" s="19" t="n">
+          <t>TOTAL DE HORAS-HOMEM PREVISTAS (HH/mês)</t>
+        </is>
+      </c>
+      <c r="E25" s="21" t="n">
+        <v>1980</v>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G25" s="21" t="n">
+        <v>3960</v>
+      </c>
+      <c r="H25" s="21" t="n">
+        <v>5060</v>
+      </c>
+      <c r="I25" s="21" t="n">
         <v>3740</v>
       </c>
-      <c r="I25" s="19" t="n">
-        <v>3520</v>
-      </c>
-      <c r="J25" s="19" t="n">
-        <v>3520</v>
+      <c r="J25" s="21" t="n">
+        <v>4840</v>
+      </c>
+      <c r="K25" s="22" t="n">
+        <v>102</v>
+      </c>
+      <c r="L25" s="23" t="n">
+        <v>22440</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J2"/>
-    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A1:L2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>